<commit_message>
update: Final artifacts, screenshots, and 60 test cases
</commit_message>
<xml_diff>
--- a/Manual Test Cases for Option 2.xlsx
+++ b/Manual Test Cases for Option 2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1992,6 +1992,1014 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Pos_037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Document conversion</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Convert a PDF to a Word document (.docx).</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>The system should output a valid, editable Word file.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>File converted successfully with editable text.</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Neg_038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>PDF editing</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Attempt to edit a PDF that is 'Read-Only' or restricted.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>The system should inform the user about the restriction.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>System failed to open the file but gave no specific error.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Assumed permission check for PDF editing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Pos_039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Image resizing</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Resize a high-resolution image (4K) to 1080p.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>The image quality should remain high despite the resize.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Image resized with minimal quality loss.</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Neg_040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Cropping</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Select a crop area completely outside the image frame.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>The system should reset the selection to the image bounds.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Selection was ignored.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Pos_041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Compression</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Use the 'Extreme Compression' setting if available.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>File size should be significantly reduced (e.g. &gt;70%).</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>File size reduced by 75%.</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Neg_042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Image format conversion</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Try to convert a file with an unsupported extension (e.g., .exe).</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>The system should reject the file immediately.</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Error message: 'Invalid file type' appeared.</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Pos_043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Meme generation</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Adjust the font size of the meme text to its maximum value.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Text should fit within the preview or scale properly.</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Text scaled but some parts were cut off.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Assumed text wrapping or scaling bounds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Pos_044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Color picker</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Copy the HEX code to clipboard using the 'Copy' button.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>The HEX code should be available in the system clipboard.</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Clipboard updated correctly.</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Pos_045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Image rotation</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Rotate an image 180° (two 90° turns).</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>The image should be upside down in the preview.</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Image rotated 180 degrees correctly.</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Neg_046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Image flipping</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Interact with the flip tool before any image is uploaded.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>The buttons should be disabled or unresponsive.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Buttons were clickable but had no effect.</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Neg_047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Document conversion</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Upload a file with a name containing special characters (e.g., !@#$%^&amp;*).</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>The system should handle the filename without crashing.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>System handled the file correctly.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Pos_048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>PDF editing</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Merge multiple PDFs (more than 5 files).</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>A single PDF containing all pages in sequence should be generated.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Merge successful for 6 files.</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Neg_049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Image resizing</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Set both width and height to 1 pixel.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>The system should allow the resize or show a minimum limit.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Image resized to 1x1 successfully.</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Pos_050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Compression</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Check the 'Preview' of the compressed image before downloading.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>The preview should reflect the quality after compression.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Preview matched the compressed output.</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Pos_051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Image format conversion</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Convert a PNG image to WebP format.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>The system should provide a WebP file for download.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Conversion successful.</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Neg_052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Meme generation</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Try to save a meme with no text and no image.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>The system should prevent saving or show a message.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Save was disabled.</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Pos_053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Color picker</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Pick a color from a semi-transparent region.</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>The system should return the calculated composite color.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Color returned correctly.</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Neg_054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Image rotation</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Set rotation angle to 0.5 degrees (if custom input exists).</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>The system should handle float values or round them.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>System rounded to 1 degree.</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Pos_055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Image flipping</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Flip a vertical image horizontally.</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>The image content should be mirrored.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Flipped correctly.</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Neg_056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Document conversion</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Try to convert a file that was deleted locally after selection.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>The system should show a 'File not found' or upload error.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>System showed upload failed.</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Pos_057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>PDF editing</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Delete a specific page from a 10-page PDF.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>The resulting PDF should have exactly 9 pages.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Page deleted successfully.</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Neg_058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Image resizing</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Upload an image with 0.01MB size (very small).</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>The system should handle small files without error.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Handled correctly.</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Pos_059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Cropping</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Use the 'Reset' button to clear crop selection.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>The selection box should disappear.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Selection reset successfully.</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Neg_060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>PixelsSuite</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Compression</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Upload a text file renamed to .png for compression.</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>The system should identify the invalid image data.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Showed 'Invalid Image'.</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>